<commit_message>
test: add comprehensive tests for budget endpoint and route optimisation
- Added Jest + Supertest tests for POST /api/route/budget
- Covered happy path, over budget, and missing country scenarios
- Added validation tests for invalid input, missing origin city, and invalid match IDs
- Verified cost breakdown correctness (ticket, flight, accommodation)
- Tested edge cases including missing flight routes and exact budget boundary
- Added unit tests for NearestNeighbourStrategy (happy path, empty input, single match)

All tests passing successfully
</commit_message>
<xml_diff>
--- a/documentation/Unit Tests/Unit Tests.xlsx
+++ b/documentation/Unit Tests/Unit Tests.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\JOBS\unosquare\worldcup-route-planner-Unosquare-RyanDonnelly\documentation\Unit Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6CE9A3B-8C31-439C-9410-30AF160B5859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E22125D-0102-4D0A-88CD-E9B38E132199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{99881518-8351-4F7A-AA61-769C163F28C7}"/>
+    <workbookView xWindow="3525" yWindow="1455" windowWidth="21600" windowHeight="11385" xr2:uid="{99881518-8351-4F7A-AA61-769C163F28C7}"/>
   </bookViews>
   <sheets>
-    <sheet name="NearestNeighbourStrategy" sheetId="1" r:id="rId1"/>
+    <sheet name="Budget" sheetId="2" r:id="rId1"/>
+    <sheet name="NearestNeighbourStrategy" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="65">
   <si>
     <t>Test ID</t>
   </si>
@@ -102,6 +103,135 @@
   </si>
   <si>
     <t>Pass</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Happy Path (Valid Route)</t>
+  </si>
+  <si>
+    <t>Valid matches covering all 3 countries within budget</t>
+  </si>
+  <si>
+    <t>Valid matchIds, valid originCityId, high budget</t>
+  </si>
+  <si>
+    <t>200 OK, feasible = true, costs calculated</t>
+  </si>
+  <si>
+    <t>Over Budget</t>
+  </si>
+  <si>
+    <t>Total cost exceeds budget</t>
+  </si>
+  <si>
+    <t>Valid matchIds, low budget</t>
+  </si>
+  <si>
+    <t>200 OK, feasible = false, suggestion about reducing cost</t>
+  </si>
+  <si>
+    <t>Missing Countries</t>
+  </si>
+  <si>
+    <t>Route does not include all required countries</t>
+  </si>
+  <si>
+    <t>Matches from only one country</t>
+  </si>
+  <si>
+    <t>200 OK, feasible = false, missingCountries populated</t>
+  </si>
+  <si>
+    <t>T4</t>
+  </si>
+  <si>
+    <t>Invalid Input</t>
+  </si>
+  <si>
+    <t>Invalid request body (empty matchIds, invalid budget)</t>
+  </si>
+  <si>
+    <t>Empty matchIds, null budget</t>
+  </si>
+  <si>
+    <t>400 Bad Request, error message returned</t>
+  </si>
+  <si>
+    <t>T5</t>
+  </si>
+  <si>
+    <t>Cost Breakdown Correctness</t>
+  </si>
+  <si>
+    <t>Ensure total cost = sum of components</t>
+  </si>
+  <si>
+    <t>Valid single match</t>
+  </si>
+  <si>
+    <t>totalCost = ticket + flight + accommodation</t>
+  </si>
+  <si>
+    <t>T6</t>
+  </si>
+  <si>
+    <t>Origin City Not Found</t>
+  </si>
+  <si>
+    <t>Invalid origin city provided</t>
+  </si>
+  <si>
+    <t>Invalid originCityId</t>
+  </si>
+  <si>
+    <t>404 Not Found, error message returned</t>
+  </si>
+  <si>
+    <t>T7</t>
+  </si>
+  <si>
+    <t>Matches Not Found</t>
+  </si>
+  <si>
+    <t>Invalid match IDs provided</t>
+  </si>
+  <si>
+    <t>Invalid matchIds</t>
+  </si>
+  <si>
+    <t>T8</t>
+  </si>
+  <si>
+    <t>Missing Flight Route</t>
+  </si>
+  <si>
+    <t>No flight exists between cities</t>
+  </si>
+  <si>
+    <t>Valid matchIds, uncommon route</t>
+  </si>
+  <si>
+    <t>200 OK, flight cost defaults to 0</t>
+  </si>
+  <si>
+    <t>T9</t>
+  </si>
+  <si>
+    <t>Exact Budget Boundary</t>
+  </si>
+  <si>
+    <t>Total cost equals budget exactly</t>
+  </si>
+  <si>
+    <t>Budget = totalCost</t>
+  </si>
+  <si>
+    <t>200 OK, feasible = true</t>
+  </si>
+  <si>
+    <t>Passed</t>
   </si>
 </sst>
 </file>
@@ -472,6 +602,222 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB70DBA0-D29A-44A2-8A85-F0DE2DF4128B}">
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="51" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" t="s">
+        <v>57</v>
+      </c>
+      <c r="E9" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{230CE8B6-53FE-4D58-823A-0F48454733BF}">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>